<commit_message>
Updated testing to accomodate assumption changes
</commit_message>
<xml_diff>
--- a/inputs/FundAssumptions.xlsx
+++ b/inputs/FundAssumptions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Software Projects\illiquid-alternative-asset-fund-model\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67662685-13DA-44F0-A332-55989E7EA8BB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99EE7FDF-F0CA-484A-A4A0-807DC5164F48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{9334B90D-CB79-461B-A22D-00B2DD3365E6}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Fund Assumptions" sheetId="3" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Fund Assumptions'!$A$1:$AL$20</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Fund Assumptions'!$A$1:$AL$19</definedName>
     <definedName name="Units">#REF!</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
@@ -40,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="140" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="61">
   <si>
     <t>Investment Name</t>
   </si>
@@ -224,9 +224,6 @@
   </si>
   <si>
     <t>Fund P</t>
-  </si>
-  <si>
-    <t>Fund X</t>
   </si>
 </sst>
 </file>
@@ -679,7 +676,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{04779175-7FD7-4891-A7A1-2B717FDD23C1}">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:AL50"/>
+  <dimension ref="A1:AL49"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="17.5703125" bestFit="1" customWidth="1"/>
@@ -1928,83 +1925,19 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
-        <v>61</v>
-      </c>
-      <c r="B18" s="4">
-        <v>250000000</v>
-      </c>
-      <c r="C18" s="4">
-        <v>78</v>
-      </c>
-      <c r="D18" s="4">
-        <v>102430077.03</v>
-      </c>
-      <c r="E18" s="9">
-        <v>46568</v>
-      </c>
-      <c r="F18" s="9">
-        <v>46934</v>
-      </c>
-      <c r="G18" s="9">
-        <v>47664</v>
-      </c>
-      <c r="H18" s="4">
-        <v>102430077.03</v>
-      </c>
-      <c r="I18" s="10">
-        <v>0.16500000000000001</v>
-      </c>
-      <c r="J18" s="11">
-        <v>0.08</v>
-      </c>
-      <c r="K18" s="12">
-        <v>0.85</v>
-      </c>
-      <c r="L18" s="11">
-        <v>7.4999999999999997E-3</v>
-      </c>
-      <c r="M18" s="13" t="b">
-        <v>0</v>
-      </c>
-      <c r="N18" s="14">
-        <v>0.12</v>
-      </c>
-      <c r="O18" s="14">
-        <v>0.08</v>
-      </c>
-      <c r="P18" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="Q18" s="15">
-        <v>5</v>
-      </c>
-      <c r="R18" s="16">
-        <f t="shared" ref="R18" si="0">+(J18-M18)*(1-O18)</f>
-        <v>7.3599999999999999E-2</v>
-      </c>
-      <c r="S18" s="17" t="s">
-        <v>21</v>
-      </c>
-      <c r="T18" s="18" t="s">
-        <v>31</v>
-      </c>
-      <c r="U18" s="18" t="s">
-        <v>32</v>
-      </c>
-      <c r="V18" s="18" t="s">
-        <v>24</v>
-      </c>
+    <row r="20" spans="1:38" x14ac:dyDescent="0.25">
+      <c r="C20" s="5"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="7"/>
     </row>
     <row r="21" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="C21" s="5"/>
+      <c r="C21" s="6"/>
       <c r="E21" s="7"/>
       <c r="F21" s="7"/>
       <c r="G21" s="7"/>
     </row>
     <row r="22" spans="1:38" x14ac:dyDescent="0.25">
-      <c r="C22" s="6"/>
       <c r="E22" s="7"/>
       <c r="F22" s="7"/>
       <c r="G22" s="7"/>
@@ -2076,8 +2009,6 @@
     </row>
     <row r="36" spans="5:7" x14ac:dyDescent="0.25">
       <c r="E36" s="7"/>
-      <c r="F36" s="7"/>
-      <c r="G36" s="7"/>
     </row>
     <row r="37" spans="5:7" x14ac:dyDescent="0.25">
       <c r="E37" s="7"/>
@@ -2117,9 +2048,6 @@
     </row>
     <row r="49" spans="5:5" x14ac:dyDescent="0.25">
       <c r="E49" s="7"/>
-    </row>
-    <row r="50" spans="5:5" x14ac:dyDescent="0.25">
-      <c r="E50" s="7"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>